<commit_message>
DBS4 28 Sep review: add the King White push on the King terms that need it
King joins B4's focus only where the push is needed and fundable:
Bamboo Sheets King pushed now (TOS $6.41 -> $7.08 market bound,
budget $73/day, checkpoint 12 Oct); Bamboo Sheets King Size queued
behind a mix fix. Every other King term stays in maintenance, with
the reason stated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
+++ b/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
@@ -1927,25 +1927,22 @@
         <v>6.41</v>
       </c>
       <c r="AS8" t="n">
-        <v>6.03</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>6.03</v>
+        <v>7.08</v>
       </c>
       <c r="AU8" t="n">
         <v>1.88</v>
       </c>
       <c r="AV8" t="n">
-        <v>221</v>
+        <v>277</v>
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>SHORT OF TARGET (22 vs 8)</t>
+          <t>KING WHITE PUSH — funded (22 → 8)</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>maintenance: top of search at the ceiling $6.03, no premium — push conditions missing: velocity</t>
+          <t>top of search 6.41 → 7.08 this write (target 7.08, market bound); base 1.88 held; budget $54 → $73/day; read 2026-10-05, checkpoint 2026-10-12</t>
         </is>
       </c>
       <c r="AY8" t="inlineStr"/>
@@ -2303,16 +2300,13 @@
         <v>4.97</v>
       </c>
       <c r="AS10" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>3.97</v>
+        <v>4.96</v>
       </c>
       <c r="AU10" t="n">
         <v>1.2</v>
       </c>
       <c r="AV10" t="n">
-        <v>231</v>
+        <v>313</v>
       </c>
       <c r="AW10" t="inlineStr">
         <is>
@@ -2321,7 +2315,7 @@
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>distribution fix first and only: cut the base, re-solve the modifier to hold the top-of-search price; no climb, no budget move</t>
+          <t>distribution fix first: base 1.60 → 1.20, top of search held at 4.96 (queued for the King push, so not descended); push entry when top of search carries ≥70% of clicks for 7 days</t>
         </is>
       </c>
       <c r="AY10" t="inlineStr">
@@ -2331,7 +2325,7 @@
       </c>
       <c r="AZ10" t="inlineStr">
         <is>
-          <t>RUN PRICE: the run takes top of search 4.96 → 4.97; the framework read gives 3.97 | SEARCH TERM: “bamboo sheets king size” — 12 of its 162 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (10), bamboo sheets california king-[Bamboo|Ca (1), Bamboo Sheets-(VHSV)-Broad-(DISC)-DO-BAM (1)</t>
+          <t>SEARCH TERM: “bamboo sheets king size” — 12 of its 162 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (10), bamboo sheets california king-[Bamboo|Ca (1), Bamboo Sheets-(VHSV)-Broad-(DISC)-DO-BAM (1)</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">

</xml_diff>

<commit_message>
DBS4 28 Sep review: count reserved units as sellable
King White has 1,759 sellable units, so the engine's RED-hero flag is
wrong. Twin White has 154 reserved (about 162 days of cover) and is
Twin's best seller, so Twin ranking stays on White instead of moving
to Navy Blue.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
+++ b/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -4629,12 +4629,12 @@
       </c>
       <c r="AZ23" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days))</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="BA23" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
+          <t>advertise BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -5382,12 +5382,12 @@
       </c>
       <c r="AZ27" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-WHITE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days)) | RUN PRICE: the run takes top of search 7.51 → 7.48; the framework read gives 3.75 | SEARCH TERM: “twin cooling sheets” — 7 of its 24 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (7)</t>
+          <t>RUN PRICE: the run takes top of search 7.51 → 7.48; the framework read gives 3.75 | SEARCH TERM: “twin cooling sheets” — 7 of its 24 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (7)</t>
         </is>
       </c>
       <c r="BA27" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE | negative-exact “twin cooling sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
+          <t>negative-exact “twin cooling sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5904,12 +5904,12 @@
       </c>
       <c r="AZ30" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days)) | RUN: swaps this campaign BAMBOO-TWIN-WHITE → BAMBOO-TWIN-BURGUNDY-NEW; the ranking SKU for the size is BAMBOO-TWIN-NAVYBLUE | SEARCH TERM: “bamboo sheets twin” — 4 of its 25 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (4)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE | RUN: swaps this campaign BAMBOO-TWIN-WHITE → BAMBOO-TWIN-BURGUNDY-NEW; the ranking SKU for the size is BAMBOO-TWIN-WHITE | SEARCH TERM: “bamboo sheets twin” — 4 of its 25 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (4)</t>
         </is>
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE | negative-exact “bamboo sheets twin” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
+          <t>advertise BAMBOO-TWIN-WHITE | negative-exact “bamboo sheets twin” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6137,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -6277,12 +6277,12 @@
       </c>
       <c r="AZ32" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days)) | SEARCH TERM: “twin bamboo sheets” — 3 of its 41 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (3)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE | SEARCH TERM: “twin bamboo sheets” — 3 of its 41 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (3)</t>
         </is>
       </c>
       <c r="BA32" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE | negative-exact “twin bamboo sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
+          <t>advertise BAMBOO-TWIN-WHITE | negative-exact “twin bamboo sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
         </is>
       </c>
     </row>
@@ -23814,7 +23814,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -23947,12 +23947,12 @@
       <c r="AY134" t="inlineStr"/>
       <c r="AZ134" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days))</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="BA134" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
+          <t>advertise BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
     </row>
@@ -24340,7 +24340,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -24464,12 +24464,12 @@
       <c r="AY137" t="inlineStr"/>
       <c r="AZ137" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days))</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="BA137" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
+          <t>advertise BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
     </row>
@@ -34285,7 +34285,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -34379,12 +34379,12 @@
       <c r="AY204" t="inlineStr"/>
       <c r="AZ204" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days))</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="BA204" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
+          <t>advertise BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
     </row>
@@ -34426,7 +34426,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -34520,12 +34520,12 @@
       <c r="AY205" t="inlineStr"/>
       <c r="AZ205" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has none available until 16 Oct; Navy Blue is the next seller with healthy stock (81 days))</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="BA205" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
+          <t>advertise BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
     </row>
@@ -43102,7 +43102,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I275" t="inlineStr"/>
@@ -44131,7 +44131,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I284" t="inlineStr"/>
@@ -44571,7 +44571,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I288" t="inlineStr"/>
@@ -44675,7 +44675,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I289" t="inlineStr"/>
@@ -45383,7 +45383,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I296" t="inlineStr"/>
@@ -45491,7 +45491,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-NAVYBLUE</t>
+          <t>BAMBOO-TWIN-WHITE</t>
         </is>
       </c>
       <c r="I297" t="inlineStr"/>

</xml_diff>

<commit_message>
DBS4 28 Sep review: judge PPC on Available stock only
Applies the reserved-inventory guideline: customer orders are never
stock, and FC transfers and processing count only for replenishment.
King White has 29 days Available, so the push stands. Twin White has
0 Available (154 FC transfers), so Twin ranking goes back to Navy
Blue. A new stock section lists the six campaigns on children with
under 5 days Available.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
+++ b/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
@@ -1069,7 +1069,7 @@
       </c>
       <c r="AZ3" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN PRICE: the run takes top of search 6.69 → 8.37; the framework read gives 6.04 | SEARCH TERM: “bamboo sheets queen size” — 52 of its 194 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (25), bamboo sheets queen size-[Bamboo|Queen]- (19), 100 Bamboo-(VLSV)-Broad-(Discovery)-DO-B (5)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN PRICE: the run takes top of search 6.69 → 8.37; the framework read gives 6.04 | SEARCH TERM: “bamboo sheets queen size” — 52 of its 194 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (25), bamboo sheets queen size-[Bamboo|Queen]- (19), 100 Bamboo-(VLSV)-Broad-(Discovery)-DO-B (5)</t>
         </is>
       </c>
       <c r="BA3" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="AZ5" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | SEARCH TERM: “bamboo sheets queen” — 7 of its 215 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (7)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | SEARCH TERM: “bamboo sheets queen” — 7 of its 215 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (7)</t>
         </is>
       </c>
       <c r="BA5" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="AZ6" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN PRICE: the run takes top of search 7.61 → 8.26; the framework read gives 3.80 | SEARCH TERM: “bamboo cooling sheets” — 18 of its 109 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (16), bamboo sheets queen size-[Bamboo|Queen]- (2)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN PRICE: the run takes top of search 7.61 → 8.26; the framework read gives 3.80 | SEARCH TERM: “bamboo cooling sheets” — 18 of its 109 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (16), bamboo sheets queen size-[Bamboo|Queen]- (2)</t>
         </is>
       </c>
       <c r="BA6" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="AZ9" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA9" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="AZ11" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | SEARCH TERM: “cooling sheets queen” — 13 of its 171 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (10), 100 Bamboo-(VLSV)-Broad-(Discovery)-DO-B (2), Cooling Sheets-[Cooling]-(VHSV)-Broad-(R (1)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | SEARCH TERM: “cooling sheets queen” — 13 of its 171 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (10), 100 Bamboo-(VLSV)-Broad-(Discovery)-DO-B (2), Cooling Sheets-[Cooling]-(VHSV)-Broad-(R (1)</t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="AZ21" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | RUN PRICE: the run takes top of search 9.10 → 8.45; the framework read gives 4.55</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | RUN PRICE: the run takes top of search 9.10 → 8.45; the framework read gives 4.55</t>
         </is>
       </c>
       <c r="BA21" t="inlineStr">
@@ -4414,26 +4414,14 @@
       <c r="AR22" t="n">
         <v>2.67</v>
       </c>
-      <c r="AS22" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="AT22" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="AU22" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="AV22" t="n">
-        <v>124</v>
-      </c>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>NOT A RANKING CAMPAIGN IN PRACTICE — top of search 6%</t>
+          <t>STOCK THROTTLE — 0 available (0.0 days); 10 reserved are FC transfers</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr">
         <is>
-          <t>distribution fix first and only: cut the base, re-solve the modifier to hold the top-of-search price; no climb, no budget move</t>
+          <t>pause until the transfers show as Available</t>
         </is>
       </c>
       <c r="AY22" t="inlineStr">
@@ -4441,11 +4429,7 @@
           <t>tos 86→147 | bid 1.43→1.08 | child BAMBOO-QUEEN-PURPLE→BAMBOO-FULL-PURPLE</t>
         </is>
       </c>
-      <c r="AZ22" t="inlineStr">
-        <is>
-          <t>RUN PRICE: the run takes top of search 2.66 → 2.67; the framework read gives 2.40</t>
-        </is>
-      </c>
+      <c r="AZ22" t="inlineStr"/>
       <c r="BA22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -4486,7 +4470,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -4629,12 +4613,12 @@
       </c>
       <c r="AZ23" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White)</t>
         </is>
       </c>
       <c r="BA23" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
     </row>
@@ -5163,23 +5147,14 @@
       <c r="AR26" t="n">
         <v>2.03</v>
       </c>
-      <c r="AS26" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AU26" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AV26" t="n">
-        <v>192</v>
-      </c>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>LEAKING — product pages 63%</t>
+          <t>STOCKOUT RISK — 0 available (0.0 days); reserved is customer orders or nothing</t>
         </is>
       </c>
       <c r="AX26" t="inlineStr">
         <is>
-          <t>distribution fix: base toward the product-page ceiling, modifier re-solved so top of search holds</t>
+          <t>cut hard: stop advertising BAMBOO-FULL-WHITE; re-point to BAMBOO-FULL-OLIVE</t>
         </is>
       </c>
       <c r="AY26" t="inlineStr">
@@ -5189,7 +5164,7 @@
       </c>
       <c r="AZ26" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-WHITE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days) | RUN: swaps this campaign BAMBOO-FULL-WHITE → BAMBOO-FULL-LIGHTOLIVE; the ranking SKU for the size is BAMBOO-FULL-OLIVE | SEARCH TERM: “cooling sheets full” — 2 of its 21 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (1), DECOLURE - B4 - QUEEN OLIVE - PRIME CAMP (1)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-WHITE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available) | RUN: swaps this campaign BAMBOO-FULL-WHITE → BAMBOO-FULL-LIGHTOLIVE; the ranking SKU for the size is BAMBOO-FULL-OLIVE | SEARCH TERM: “cooling sheets full” — 2 of its 21 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (1), DECOLURE - B4 - QUEEN OLIVE - PRIME CAMP (1)</t>
         </is>
       </c>
       <c r="BA26" t="inlineStr">
@@ -5236,7 +5211,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -5353,26 +5328,14 @@
       <c r="AR27" t="n">
         <v>7.48</v>
       </c>
-      <c r="AS27" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="AT27" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="AU27" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="AV27" t="n">
-        <v>297</v>
-      </c>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>LEAKING — product pages 62%</t>
+          <t>STOCK THROTTLE — 0 available (0.0 days); 154 reserved are FC transfers</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr">
         <is>
-          <t>distribution fix: base toward the product-page ceiling, modifier re-solved so top of search holds</t>
+          <t>stop advertising BAMBOO-TWIN-WHITE here; re-point to BAMBOO-TWIN-NAVYBLUE, which has Available stock; back to BAMBOO-TWIN-WHITE once the transfers show as Available</t>
         </is>
       </c>
       <c r="AY27" t="inlineStr">
@@ -5382,12 +5345,12 @@
       </c>
       <c r="AZ27" t="inlineStr">
         <is>
-          <t>RUN PRICE: the run takes top of search 7.51 → 7.48; the framework read gives 3.75 | SEARCH TERM: “twin cooling sheets” — 7 of its 24 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (7)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-WHITE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White) | SEARCH TERM: “twin cooling sheets” — 7 of its 24 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (7)</t>
         </is>
       </c>
       <c r="BA27" t="inlineStr">
         <is>
-          <t>negative-exact “twin cooling sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE | negative-exact “twin cooling sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5727,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5904,12 +5867,12 @@
       </c>
       <c r="AZ30" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE | RUN: swaps this campaign BAMBOO-TWIN-WHITE → BAMBOO-TWIN-BURGUNDY-NEW; the ranking SKU for the size is BAMBOO-TWIN-WHITE | SEARCH TERM: “bamboo sheets twin” — 4 of its 25 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (4)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White) | RUN: swaps this campaign BAMBOO-TWIN-WHITE → BAMBOO-TWIN-BURGUNDY-NEW; the ranking SKU for the size is BAMBOO-TWIN-NAVYBLUE | SEARCH TERM: “bamboo sheets twin” — 4 of its 25 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (4)</t>
         </is>
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE | negative-exact “bamboo sheets twin” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE | negative-exact “bamboo sheets twin” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6100,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -6277,12 +6240,12 @@
       </c>
       <c r="AZ32" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE | SEARCH TERM: “twin bamboo sheets” — 3 of its 41 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (3)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White) | SEARCH TERM: “twin bamboo sheets” — 3 of its 41 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (3)</t>
         </is>
       </c>
       <c r="BA32" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE | negative-exact “twin bamboo sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE | negative-exact “twin bamboo sheets” in LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6547,7 @@
       </c>
       <c r="AZ34" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | SEARCH TERM: “bamboo deep pocket queen sheets” — 1 of its 12 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (1)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | SEARCH TERM: “bamboo deep pocket queen sheets” — 1 of its 12 clicks (30d) go to LTSF-ALL-Broad-(Clearance)-DO-AGED-ALL (1)</t>
         </is>
       </c>
       <c r="BA34" t="inlineStr">
@@ -9125,7 +9088,7 @@
       </c>
       <c r="AZ48" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA48" t="inlineStr">
@@ -11636,7 +11599,7 @@
       </c>
       <c r="AZ62" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN PRICE: the run takes top of search 4.99 → 5.54; the framework read gives 4.99</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN PRICE: the run takes top of search 4.99 → 5.54; the framework read gives 4.99</t>
         </is>
       </c>
       <c r="BA62" t="inlineStr">
@@ -12324,7 +12287,7 @@
       <c r="AY66" t="inlineStr"/>
       <c r="AZ66" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA66" t="inlineStr">
@@ -13356,7 +13319,7 @@
       </c>
       <c r="AZ72" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA72" t="inlineStr">
@@ -14042,7 +14005,7 @@
       </c>
       <c r="AZ76" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN PRICE: the run takes top of search 2.67 → 2.96; the framework read gives 3.47</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN PRICE: the run takes top of search 2.67 → 2.96; the framework read gives 3.47</t>
         </is>
       </c>
       <c r="BA76" t="inlineStr">
@@ -14411,7 +14374,7 @@
       </c>
       <c r="AZ78" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 7.3 top-of-search clicks/day; winning every auction at today’s volume would give ~2.3 — the requirement is above what the auction holds</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 7.3 top-of-search clicks/day; winning every auction at today’s volume would give ~2.3 — the requirement is above what the auction holds</t>
         </is>
       </c>
       <c r="BA78" t="inlineStr">
@@ -16771,7 +16734,7 @@
       </c>
       <c r="AZ92" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA92" t="inlineStr">
@@ -17284,7 +17247,7 @@
       </c>
       <c r="AZ95" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 14.7 top-of-search clicks/day; winning every auction at today’s volume would give ~6.5 — the requirement is above what the auction holds</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 14.7 top-of-search clicks/day; winning every auction at today’s volume would give ~6.5 — the requirement is above what the auction holds</t>
         </is>
       </c>
       <c r="BA95" t="inlineStr">
@@ -17795,7 +17758,7 @@
       <c r="AY98" t="inlineStr"/>
       <c r="AZ98" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA98" t="inlineStr">
@@ -18492,7 +18455,7 @@
       </c>
       <c r="AZ102" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 5.3 top-of-search clicks/day; winning every auction at today’s volume would give ~1.4 — the requirement is above what the auction holds</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 5.3 top-of-search clicks/day; winning every auction at today’s volume would give ~1.4 — the requirement is above what the auction holds</t>
         </is>
       </c>
       <c r="BA102" t="inlineStr">
@@ -19007,7 +18970,7 @@
       <c r="AY105" t="inlineStr"/>
       <c r="AZ105" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | TRAFFIC: needs 5.3 top-of-search clicks/day; winning every auction at today’s volume would give ~2.0 — the requirement is above what the auction holds</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | TRAFFIC: needs 5.3 top-of-search clicks/day; winning every auction at today’s volume would give ~2.0 — the requirement is above what the auction holds</t>
         </is>
       </c>
       <c r="BA105" t="inlineStr">
@@ -19191,7 +19154,7 @@
       </c>
       <c r="AZ106" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 6.1 top-of-search clicks/day; winning every auction at today’s volume would give ~2.0 — the requirement is above what the auction holds</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | TRAFFIC: needs 6.1 top-of-search clicks/day; winning every auction at today’s volume would give ~2.0 — the requirement is above what the auction holds</t>
         </is>
       </c>
       <c r="BA106" t="inlineStr">
@@ -19540,7 +19503,7 @@
       </c>
       <c r="AZ108" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA108" t="inlineStr">
@@ -19724,7 +19687,7 @@
       </c>
       <c r="AZ109" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA109" t="inlineStr">
@@ -19893,7 +19856,7 @@
       </c>
       <c r="AZ110" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | KEYWORD: “cool sheets for hot sleepers” is also bought exact by DBS4-SP-Cooling Sheets For Hot Sleepers-[Cooling]-(LSV)-Exac — one owner per term; keep the one on the ranking SKU, pause the other</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | KEYWORD: “cool sheets for hot sleepers” is also bought exact by DBS4-SP-Cooling Sheets For Hot Sleepers-[Cooling]-(LSV)-Exac — one owner per term; keep the one on the ranking SKU, pause the other</t>
         </is>
       </c>
       <c r="BA110" t="inlineStr">
@@ -20750,7 +20713,7 @@
       </c>
       <c r="AZ115" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA115" t="inlineStr">
@@ -21104,7 +21067,7 @@
       <c r="AY117" t="inlineStr"/>
       <c r="AZ117" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA117" t="inlineStr">
@@ -21781,7 +21744,7 @@
       <c r="AY121" t="inlineStr"/>
       <c r="AZ121" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA121" t="inlineStr">
@@ -22939,7 +22902,7 @@
       <c r="AY128" t="inlineStr"/>
       <c r="AZ128" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA128" t="inlineStr">
@@ -23104,7 +23067,7 @@
       <c r="AY129" t="inlineStr"/>
       <c r="AZ129" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA129" t="inlineStr">
@@ -23581,23 +23544,14 @@
       <c r="AQ132" t="n">
         <v>2.61</v>
       </c>
-      <c r="AS132" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="AU132" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV132" t="n">
-        <v>161</v>
-      </c>
       <c r="AW132" t="inlineStr">
         <is>
-          <t>LEAKING — product pages 29%</t>
+          <t>STOCKOUT RISK — 0 available (0.0 days); reserved is customer orders or nothing</t>
         </is>
       </c>
       <c r="AX132" t="inlineStr">
         <is>
-          <t>distribution fix: base toward the product-page ceiling, modifier re-solved so top of search holds</t>
+          <t>cut hard: stop advertising BAMBOO-FULL-WHITE; re-point to BAMBOO-FULL-OLIVE</t>
         </is>
       </c>
       <c r="AY132" t="inlineStr">
@@ -23607,7 +23561,7 @@
       </c>
       <c r="AZ132" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-WHITE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days) | RUN: swaps this campaign BAMBOO-FULL-WHITE → BAMBOO-FULL-LIGHTOLIVE; the ranking SKU for the size is BAMBOO-FULL-OLIVE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-WHITE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available) | RUN: swaps this campaign BAMBOO-FULL-WHITE → BAMBOO-FULL-LIGHTOLIVE; the ranking SKU for the size is BAMBOO-FULL-OLIVE</t>
         </is>
       </c>
       <c r="BA132" t="inlineStr">
@@ -23814,7 +23768,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -23947,12 +23901,12 @@
       <c r="AY134" t="inlineStr"/>
       <c r="AZ134" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White)</t>
         </is>
       </c>
       <c r="BA134" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
     </row>
@@ -24293,7 +24247,7 @@
       </c>
       <c r="AZ136" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA136" t="inlineStr">
@@ -24340,7 +24294,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -24464,12 +24418,12 @@
       <c r="AY137" t="inlineStr"/>
       <c r="AZ137" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-BURGUNDY-NEW; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White)</t>
         </is>
       </c>
       <c r="BA137" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
     </row>
@@ -24641,7 +24595,7 @@
       <c r="AY138" t="inlineStr"/>
       <c r="AZ138" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA138" t="inlineStr">
@@ -25082,7 +25036,7 @@
       </c>
       <c r="AZ141" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA141" t="inlineStr">
@@ -25222,32 +25176,20 @@
       <c r="AQ142" t="n">
         <v>5.51</v>
       </c>
-      <c r="AS142" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="AT142" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="AU142" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AV142" t="n">
-        <v>82</v>
-      </c>
       <c r="AW142" t="inlineStr">
         <is>
-          <t>NO CLICKS — on, not delivering</t>
+          <t>STOCKOUT RISK — 0 available (0.0 days); reserved is customer orders or nothing</t>
         </is>
       </c>
       <c r="AX142" t="inlineStr">
         <is>
-          <t>hold the base, move the modifier only (cutting the base of a row that is not delivering makes it worse)</t>
+          <t>cut hard: stop advertising BAMBOO-FULL-WHITE; re-point to BAMBOO-FULL-OLIVE</t>
         </is>
       </c>
       <c r="AY142" t="inlineStr"/>
       <c r="AZ142" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-WHITE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-WHITE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA142" t="inlineStr">
@@ -25687,7 +25629,7 @@
       <c r="AY145" t="inlineStr"/>
       <c r="AZ145" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA145" t="inlineStr">
@@ -25841,7 +25783,7 @@
       </c>
       <c r="AZ146" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | ROS modifier 20% not earned (framework §8: 15+ rest-of-search clicks converting at or above product pages)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | ROS modifier 20% not earned (framework §8: 15+ rest-of-search clicks converting at or above product pages)</t>
         </is>
       </c>
       <c r="BA146" t="inlineStr">
@@ -26417,7 +26359,7 @@
       <c r="AY150" t="inlineStr"/>
       <c r="AZ150" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA150" t="inlineStr">
@@ -26570,7 +26512,7 @@
       <c r="AY151" t="inlineStr"/>
       <c r="AZ151" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA151" t="inlineStr">
@@ -28468,7 +28410,7 @@
       </c>
       <c r="AZ164" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA164" t="inlineStr">
@@ -28766,7 +28708,7 @@
       <c r="AY166" t="inlineStr"/>
       <c r="AZ166" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA166" t="inlineStr">
@@ -28922,7 +28864,7 @@
       <c r="AY167" t="inlineStr"/>
       <c r="AZ167" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA167" t="inlineStr">
@@ -29525,7 +29467,7 @@
       <c r="AY171" t="inlineStr"/>
       <c r="AZ171" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA171" t="inlineStr">
@@ -29676,7 +29618,7 @@
       </c>
       <c r="AZ172" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA172" t="inlineStr">
@@ -30418,7 +30360,7 @@
       <c r="AY177" t="inlineStr"/>
       <c r="AZ177" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA177" t="inlineStr">
@@ -30735,7 +30677,7 @@
       <c r="AY179" t="inlineStr"/>
       <c r="AZ179" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA179" t="inlineStr">
@@ -30894,7 +30836,7 @@
       <c r="AY180" t="inlineStr"/>
       <c r="AZ180" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA180" t="inlineStr">
@@ -32456,7 +32398,7 @@
       </c>
       <c r="AZ191" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA191" t="inlineStr">
@@ -32601,7 +32543,7 @@
       </c>
       <c r="AZ192" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA192" t="inlineStr">
@@ -32746,7 +32688,7 @@
       </c>
       <c r="AZ193" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA193" t="inlineStr">
@@ -32899,7 +32841,7 @@
       <c r="AY194" t="inlineStr"/>
       <c r="AZ194" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA194" t="inlineStr">
@@ -33064,7 +33006,7 @@
       <c r="AY195" t="inlineStr"/>
       <c r="AZ195" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA195" t="inlineStr">
@@ -33638,7 +33580,7 @@
       </c>
       <c r="AZ199" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | ROS modifier 20% not earned (framework §8: 15+ rest-of-search clicks converting at or above product pages)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE | ROS modifier 20% not earned (framework §8: 15+ rest-of-search clicks converting at or above product pages)</t>
         </is>
       </c>
       <c r="BA199" t="inlineStr">
@@ -33940,7 +33882,7 @@
       </c>
       <c r="AZ201" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA201" t="inlineStr">
@@ -34093,7 +34035,7 @@
       <c r="AY202" t="inlineStr"/>
       <c r="AZ202" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA202" t="inlineStr">
@@ -34285,7 +34227,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -34379,12 +34321,12 @@
       <c r="AY204" t="inlineStr"/>
       <c r="AZ204" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White)</t>
         </is>
       </c>
       <c r="BA204" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
     </row>
@@ -34426,7 +34368,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -34520,12 +34462,12 @@
       <c r="AY205" t="inlineStr"/>
       <c r="AZ205" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-WHITE</t>
+          <t>SKU: ranking campaign advertises BAMBOO-TWIN-LIGHTBLUE; the size’s ranking SKU is BAMBOO-TWIN-NAVYBLUE (Twin White has 0 available — its 154 reserved are FC transfers, sellable in about 3–10 days; Navy Blue carries it (80 days available) until they show as Available, then back to White)</t>
         </is>
       </c>
       <c r="BA205" t="inlineStr">
         <is>
-          <t>advertise BAMBOO-TWIN-WHITE</t>
+          <t>advertise BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
     </row>
@@ -34827,7 +34769,7 @@
       <c r="AY207" t="inlineStr"/>
       <c r="AZ207" t="inlineStr">
         <is>
-          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA207" t="inlineStr">
@@ -36253,7 +36195,7 @@
       </c>
       <c r="AZ218" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | OBJECTIVE: the name says Ranking, the tag says Conversions | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | OBJECTIVE: the name says Ranking, the tag says Conversions | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA218" t="inlineStr">
@@ -37093,7 +37035,7 @@
       </c>
       <c r="AZ224" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | OBJECTIVE: the name says Ranking, the tag says Conversions | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | OBJECTIVE: the name says Ranking, the tag says Conversions | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA224" t="inlineStr">
@@ -37232,7 +37174,7 @@
       </c>
       <c r="AZ225" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA225" t="inlineStr">
@@ -37756,7 +37698,7 @@
       </c>
       <c r="AZ229" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA229" t="inlineStr">
@@ -39251,7 +39193,7 @@
       </c>
       <c r="AZ241" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA241" t="inlineStr">
@@ -40322,7 +40264,7 @@
       </c>
       <c r="AZ250" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA250" t="inlineStr">
@@ -40572,7 +40514,7 @@
       </c>
       <c r="AZ252" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA252" t="inlineStr">
@@ -41120,7 +41062,7 @@
       <c r="AY257" t="inlineStr"/>
       <c r="AZ257" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White is out until 27 Oct; Olive is the size’s top seller with 75 days)</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-FULL-LIGHTBLUE; the size’s ranking SKU is BAMBOO-FULL-OLIVE (Full White has 0 available; Olive is the size’s top seller with 70 days available)</t>
         </is>
       </c>
       <c r="BA257" t="inlineStr">
@@ -41587,7 +41529,7 @@
       <c r="AY261" t="inlineStr"/>
       <c r="AZ261" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA261" t="inlineStr">
@@ -42142,7 +42084,7 @@
       </c>
       <c r="AZ266" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days)</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-OLIVE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available)</t>
         </is>
       </c>
       <c r="BA266" t="inlineStr">
@@ -42269,7 +42211,7 @@
       </c>
       <c r="AZ267" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 23 days of cover against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 70 days) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
+          <t>OBJECTIVE: tagged Conversions but a Exact campaign is Ranking by the standard | SKU: ranking campaign advertises BAMBOO-QUEEN-WHITE; the size’s ranking SKU is BAMBOO-QUEEN-LIGHTBLUE (Queen White has 15 days Available against a 27 Oct arrival and sells on its own; Light Blue is the next seller with 57 days Available) | RUN: swaps this campaign BAMBOO-QUEEN-WHITE → BAMBOO-QUEEN-OLIVE; the ranking SKU for the size is BAMBOO-QUEEN-LIGHTBLUE</t>
         </is>
       </c>
       <c r="BA267" t="inlineStr">
@@ -43102,7 +43044,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I275" t="inlineStr"/>
@@ -44131,7 +44073,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I284" t="inlineStr"/>
@@ -44571,7 +44513,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I288" t="inlineStr"/>
@@ -44675,7 +44617,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I289" t="inlineStr"/>
@@ -44729,12 +44671,12 @@
       </c>
       <c r="AW289" t="inlineStr">
         <is>
-          <t>INSIDE ITS CEILING — ACoS 17%</t>
+          <t>STOCK THROTTLE — 0 available (0.0 days); 154 reserved are FC transfers</t>
         </is>
       </c>
       <c r="AX289" t="inlineStr">
         <is>
-          <t>hold; nothing moves, including the top-of-search modifier</t>
+          <t>keep on a lower budget (branded / proven exact only)</t>
         </is>
       </c>
       <c r="AY289" t="inlineStr"/>
@@ -45383,7 +45325,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I296" t="inlineStr"/>
@@ -45491,7 +45433,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-WHITE</t>
+          <t>BAMBOO-TWIN-NAVYBLUE</t>
         </is>
       </c>
       <c r="I297" t="inlineStr"/>

</xml_diff>

<commit_message>
DBS4/DBS6 28 Sep reviews: name the LTSF SKU for Auto, Broad and Phrase
LTSF (operator, 28 Sep) = a low-selling child with high stock: a
non-White child with 180+ days of Available cover, or 90+ days while
selling at or below its size's median. Each size's pick has the most
units beyond 90 days of cover among children still selling 5+ a
month. Deal dates confirmed: B4 ends 28 Sep, B6 ends 30 Sep.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
+++ b/docs/DBS4_Campaign_Review_20260928-9e6e6bb5.xlsx
@@ -1189,7 +1189,7 @@
       </c>
       <c r="AZ4" t="inlineStr">
         <is>
-          <t>OBJECTIVE: tagged Ranking but a Broad campaign is Discovery by the standard | SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; it should advertise an LTSF SKU (list pending) | MISSING: over its ceiling and the run does not bring the base down | SEARCH TERM: buys 1 exact ranking terms (1 clicks, $3 in 30d) — “cooling sheets queen” 1</t>
+          <t>OBJECTIVE: tagged Ranking but a Broad campaign is Discovery by the standard | SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; King has no LTSF child today — advertise a non-White child | MISSING: over its ceiling and the run does not bring the base down | SEARCH TERM: buys 1 exact ranking terms (1 clicks, $3 in 30d) — “cooling sheets queen” 1</t>
         </is>
       </c>
       <c r="BA4" t="inlineStr">
@@ -43736,7 +43736,7 @@
       </c>
       <c r="AZ279" t="inlineStr">
         <is>
-          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; it should advertise an LTSF SKU (list pending) | SEARCH TERM: buys 3 exact ranking terms (20 clicks, $36 in 30d) — “bamboo sheets” 13, “bamboo sheets queen size” 5, “cooling sheets queen” 2</t>
+          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; King has no LTSF child today — advertise a non-White child | SEARCH TERM: buys 3 exact ranking terms (20 clicks, $36 in 30d) — “bamboo sheets” 13, “bamboo sheets queen size” 5, “cooling sheets queen” 2</t>
         </is>
       </c>
       <c r="BA279" t="inlineStr">
@@ -43852,12 +43852,12 @@
       </c>
       <c r="AZ280" t="inlineStr">
         <is>
-          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-QUEEN-WHITE; it should advertise an LTSF SKU (list pending) | SEARCH TERM: buys 4 exact ranking terms (31 clicks, $86 in 30d) — “bamboo sheets queen size” 19, “bamboo sheets” 9, “bamboo cooling sheets” 2, “bamboo sheets deep pocket” 1</t>
+          <t>SKU: Broad campaign advertises BAMBOO-QUEEN-WHITE; the Queen LTSF SKU is BAMBOO-QUEEN-LIGHTOLIVE (10 sold in 30 days, 113 Available, 174 days) | SEARCH TERM: buys 4 exact ranking terms (31 clicks, $86 in 30d) — “bamboo sheets queen size” 19, “bamboo sheets” 9, “bamboo cooling sheets” 2, “bamboo sheets deep pocket” 1</t>
         </is>
       </c>
       <c r="BA280" t="inlineStr">
         <is>
-          <t>negative-exact the ranking terms it buys (they belong to their exact campaigns)</t>
+          <t>advertise BAMBOO-QUEEN-LIGHTOLIVE | negative-exact the ranking terms it buys (they belong to their exact campaigns)</t>
         </is>
       </c>
     </row>
@@ -43968,7 +43968,7 @@
       </c>
       <c r="AZ281" t="inlineStr">
         <is>
-          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; it should advertise an LTSF SKU (list pending) | MISSING: over its ceiling and the run does not bring the base down | SEARCH TERM: buys 2 exact ranking terms (2 clicks, $3 in 30d) — “bamboo sheets king” 1, “bamboo sheets king size” 1</t>
+          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; King has no LTSF child today — advertise a non-White child | MISSING: over its ceiling and the run does not bring the base down | SEARCH TERM: buys 2 exact ranking terms (2 clicks, $3 in 30d) — “bamboo sheets king” 1, “bamboo sheets king size” 1</t>
         </is>
       </c>
       <c r="BA281" t="inlineStr">
@@ -44084,12 +44084,12 @@
       </c>
       <c r="AZ282" t="inlineStr">
         <is>
-          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-CALIFKING-WHITE; it should advertise an LTSF SKU (list pending) | SEARCH TERM: buys 3 exact ranking terms (5 clicks, $11 in 30d) — “bamboo sheets” 2, “california king bamboo sheets” 2, “bamboo sheets king size” 1</t>
+          <t>SKU: Broad campaign advertises BAMBOO-CALIFKING-WHITE; the California King LTSF SKU is BAMBOO-CALIFKING-GREY (7 sold in 30 days, 56 Available, 156 days) | SEARCH TERM: buys 3 exact ranking terms (5 clicks, $11 in 30d) — “bamboo sheets” 2, “california king bamboo sheets” 2, “bamboo sheets king size” 1</t>
         </is>
       </c>
       <c r="BA282" t="inlineStr">
         <is>
-          <t>negative-exact the ranking terms it buys (they belong to their exact campaigns)</t>
+          <t>advertise BAMBOO-CALIFKING-GREY | negative-exact the ranking terms it buys (they belong to their exact campaigns)</t>
         </is>
       </c>
     </row>
@@ -44200,7 +44200,7 @@
       </c>
       <c r="AZ283" t="inlineStr">
         <is>
-          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; it should advertise an LTSF SKU (list pending) | RUN: cuts a campaign that is inside its ceiling (bid 1.3→1.17, bid 1.6→1.44) — hold instead | SEARCH TERM: buys 1 exact ranking terms (1 clicks, $2 in 30d) — “bamboo sheets california king” 1</t>
+          <t>SKU: Broad campaign advertises the White ranking SKU BAMBOO-KING-WHITE; King has no LTSF child today — advertise a non-White child | RUN: cuts a campaign that is inside its ceiling (bid 1.3→1.17, bid 1.6→1.44) — hold instead | SEARCH TERM: buys 1 exact ranking terms (1 clicks, $2 in 30d) — “bamboo sheets california king” 1</t>
         </is>
       </c>
       <c r="BA283" t="inlineStr">
@@ -44314,8 +44314,16 @@
           <t>negatives 40 term(s)→131 term(s)</t>
         </is>
       </c>
-      <c r="AZ284" t="inlineStr"/>
-      <c r="BA284" t="inlineStr"/>
+      <c r="AZ284" t="inlineStr">
+        <is>
+          <t>SKU: Auto campaign advertises BAMBOO-TWIN-NAVYBLUE; the Twin LTSF SKU is BAMBOO-TWIN-BURGUNDY-NEW (5 sold in 30 days, 133 Available, 665 days)</t>
+        </is>
+      </c>
+      <c r="BA284" t="inlineStr">
+        <is>
+          <t>advertise BAMBOO-TWIN-BURGUNDY-NEW</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -44424,7 +44432,7 @@
       </c>
       <c r="AZ285" t="inlineStr">
         <is>
-          <t>SKU: Auto campaign advertises the White ranking SKU BAMBOO-KING-WHITE; it should advertise an LTSF SKU (list pending)</t>
+          <t>SKU: Auto campaign advertises the White ranking SKU BAMBOO-KING-WHITE; King has no LTSF child today — advertise a non-White child</t>
         </is>
       </c>
       <c r="BA285" t="inlineStr"/>

</xml_diff>